<commit_message>
update analysis lobanov, ANOVA, mixedLM
</commit_message>
<xml_diff>
--- a/src/analysis/formant_results_all_vowels_model_standard.xlsx
+++ b/src/analysis/formant_results_all_vowels_model_standard.xlsx
@@ -429,140 +429,145 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>vowel_label</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>vowel_label</t>
+          <t>F1_mid_mean</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>F1_mid_mean</t>
+          <t>F2_mid_mean</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>F2_mid_mean</t>
+          <t>F1_mid_mean(z)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>F1_mid_mean(z)</t>
+          <t>F2_mid_mean(z)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>F2_mid_mean(z)</t>
+          <t>duration</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>573.2508744340857</v>
+      </c>
       <c r="C2" t="n">
-        <v>573.2508744340857</v>
+        <v>1018.915274825678</v>
       </c>
       <c r="D2" t="n">
-        <v>1018.915274825678</v>
+        <v>1.369334284817008</v>
       </c>
       <c r="E2" t="n">
-        <v>1.369334284817008</v>
+        <v>-0.535360508666695</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.535360508666695</v>
+        <v>0.1020320429175069</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ae</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>454.9736402533687</v>
+      </c>
       <c r="C3" t="n">
-        <v>454.9736402533687</v>
+        <v>1935.437596342123</v>
       </c>
       <c r="D3" t="n">
-        <v>1935.437596342123</v>
+        <v>0.319213958224415</v>
       </c>
       <c r="E3" t="n">
-        <v>0.319213958224415</v>
+        <v>0.9065967074435456</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9065967074435456</v>
+        <v>0.1284254977113663</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>i</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>340.850615615494</v>
+      </c>
       <c r="C4" t="n">
-        <v>340.850615615494</v>
+        <v>2098.134697239299</v>
       </c>
       <c r="D4" t="n">
-        <v>2098.134697239299</v>
+        <v>-0.6940233628423768</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.6940233628423768</v>
+        <v>1.16256675113079</v>
       </c>
       <c r="F4" t="n">
-        <v>1.16256675113079</v>
+        <v>0.1154647399056731</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>o</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>371.2263311600728</v>
+      </c>
       <c r="C5" t="n">
-        <v>371.2263311600728</v>
+        <v>737.7337963020947</v>
       </c>
       <c r="D5" t="n">
-        <v>737.7337963020947</v>
+        <v>-0.4243336245837088</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.4243336245837088</v>
+        <v>-0.9777410731932428</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.9777410731932428</v>
+        <v>0.09870612224862865</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>354.798083133915</v>
+      </c>
       <c r="C6" t="n">
-        <v>354.798083133915</v>
+        <v>1005.757279782782</v>
       </c>
       <c r="D6" t="n">
-        <v>1005.757279782782</v>
+        <v>-0.5701912556153401</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.5701912556153401</v>
+        <v>-0.5560618767143963</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.5560618767143963</v>
+        <v>0.08385820083527974</v>
       </c>
     </row>
   </sheetData>

</xml_diff>